<commit_message>
chore: refresh legacy email workbooks
</commit_message>
<xml_diff>
--- a/po.xlsx
+++ b/po.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -28607,7 +28607,7 @@
       </c>
       <c r="F414" t="inlineStr">
         <is>
-          <t>InReview</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="G414" t="inlineStr">
@@ -28644,18 +28644,13 @@
           <t>Contracted</t>
         </is>
       </c>
-      <c r="Q414" t="inlineStr">
-        <is>
-          <t>arman.b</t>
-        </is>
-      </c>
       <c r="R414" t="inlineStr">
         <is>
           <t>Procurement Manager</t>
         </is>
       </c>
       <c r="S414" s="5" t="n">
-        <v>46269.57989583333</v>
+        <v>46273.21885416667</v>
       </c>
     </row>
     <row r="415">
@@ -60936,7 +60931,7 @@
       </c>
       <c r="F888" t="inlineStr">
         <is>
-          <t>Confirmed</t>
+          <t>InReview</t>
         </is>
       </c>
       <c r="G888" t="inlineStr">
@@ -60956,7 +60951,7 @@
         <v>46261.5</v>
       </c>
       <c r="M888" t="n">
-        <v>390</v>
+        <v>304</v>
       </c>
       <c r="N888" t="inlineStr">
         <is>
@@ -60973,13 +60968,18 @@
           <t>Contracted</t>
         </is>
       </c>
+      <c r="Q888" t="inlineStr">
+        <is>
+          <t>Riyaz.n</t>
+        </is>
+      </c>
       <c r="R888" t="inlineStr">
         <is>
-          <t>LPO sent/shared with supplier</t>
+          <t>Procurement Manager</t>
         </is>
       </c>
       <c r="S888" s="5" t="n">
-        <v>46265.5</v>
+        <v>46273.23171296297</v>
       </c>
     </row>
     <row r="889">
@@ -63681,7 +63681,7 @@
       </c>
       <c r="F928" t="inlineStr">
         <is>
-          <t>InReview</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="G928" t="inlineStr">
@@ -63718,18 +63718,13 @@
           <t>Contracted</t>
         </is>
       </c>
-      <c r="Q928" t="inlineStr">
-        <is>
-          <t>arman.b</t>
-        </is>
-      </c>
       <c r="R928" t="inlineStr">
         <is>
-          <t>Accounting Manager</t>
+          <t>Procurement Manager</t>
         </is>
       </c>
       <c r="S928" s="5" t="n">
-        <v>46269.57782407408</v>
+        <v>46273.23692019676</v>
       </c>
     </row>
     <row r="929">
@@ -63893,7 +63888,7 @@
       </c>
       <c r="F931" t="inlineStr">
         <is>
-          <t>InReview</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="G931" t="inlineStr">
@@ -63930,18 +63925,13 @@
           <t>Contracted</t>
         </is>
       </c>
-      <c r="Q931" t="inlineStr">
-        <is>
-          <t>arman.b</t>
-        </is>
-      </c>
       <c r="R931" t="inlineStr">
         <is>
-          <t>Accounting Manager</t>
+          <t>Procurement Manager</t>
         </is>
       </c>
       <c r="S931" s="5" t="n">
-        <v>46269.5840625</v>
+        <v>46273.21885416667</v>
       </c>
     </row>
     <row r="932">
@@ -67467,7 +67457,7 @@
       </c>
       <c r="F983" t="inlineStr">
         <is>
-          <t>InReview</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="G983" t="inlineStr">
@@ -67504,18 +67494,13 @@
           <t>Contracted</t>
         </is>
       </c>
-      <c r="Q983" t="inlineStr">
-        <is>
-          <t>arman.b</t>
-        </is>
-      </c>
       <c r="R983" t="inlineStr">
         <is>
           <t>Procurement Manager</t>
         </is>
       </c>
       <c r="S983" s="5" t="n">
-        <v>46269.57989583333</v>
+        <v>46273.2256712963</v>
       </c>
     </row>
     <row r="984">
@@ -67541,7 +67526,7 @@
       </c>
       <c r="F984" t="inlineStr">
         <is>
-          <t>InReview</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="G984" t="inlineStr">
@@ -67578,18 +67563,13 @@
           <t>Contracted</t>
         </is>
       </c>
-      <c r="Q984" t="inlineStr">
-        <is>
-          <t>arman.b</t>
-        </is>
-      </c>
       <c r="R984" t="inlineStr">
         <is>
           <t>Procurement Manager</t>
         </is>
       </c>
       <c r="S984" s="5" t="n">
-        <v>46269.57989583333</v>
+        <v>46273.21885416667</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: classify requisition actions across dashboard and email
</commit_message>
<xml_diff>
--- a/po.xlsx
+++ b/po.xlsx
@@ -70160,7 +70160,7 @@
         </is>
       </c>
       <c r="S953" s="5" t="n">
-        <v>46273.57066753472</v>
+        <v>46273.57065972222</v>
       </c>
     </row>
     <row r="954">
@@ -70234,7 +70234,7 @@
         </is>
       </c>
       <c r="S954" s="5" t="n">
-        <v>46273.57066753472</v>
+        <v>46273.57065972222</v>
       </c>
     </row>
     <row r="955">
@@ -70299,16 +70299,16 @@
       </c>
       <c r="Q955" t="inlineStr">
         <is>
-          <t>Riyaz.n</t>
+          <t>arman.b</t>
         </is>
       </c>
       <c r="R955" t="inlineStr">
         <is>
-          <t>Procurement Manager</t>
+          <t>Accounting Manager</t>
         </is>
       </c>
       <c r="S955" s="5" t="n">
-        <v>46273.52849537037</v>
+        <v>46273.58289351852</v>
       </c>
     </row>
     <row r="956">
@@ -70746,7 +70746,7 @@
         </is>
       </c>
       <c r="S961" s="5" t="n">
-        <v>46273.57066753472</v>
+        <v>46273.57065972222</v>
       </c>
     </row>
     <row r="962">
@@ -70820,7 +70820,7 @@
         </is>
       </c>
       <c r="S962" s="5" t="n">
-        <v>46273.57066753472</v>
+        <v>46273.57065972222</v>
       </c>
     </row>
     <row r="963">

</xml_diff>

<commit_message>
fix: keep every requisition visible in email
</commit_message>
<xml_diff>
--- a/po.xlsx
+++ b/po.xlsx
@@ -69109,7 +69109,7 @@
       </c>
       <c r="F939" t="inlineStr">
         <is>
-          <t>InReview</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="G939" t="inlineStr">
@@ -69148,16 +69148,16 @@
       </c>
       <c r="Q939" t="inlineStr">
         <is>
-          <t>arman.b</t>
+          <t>not recorded</t>
         </is>
       </c>
       <c r="R939" t="inlineStr">
         <is>
-          <t>Accounting Manager</t>
+          <t>Procurement Manager</t>
         </is>
       </c>
       <c r="S939" s="5" t="n">
-        <v>46272.54193287037</v>
+        <v>46274.26350694444</v>
       </c>
     </row>
     <row r="940">
@@ -69523,7 +69523,7 @@
       </c>
       <c r="F945" t="inlineStr">
         <is>
-          <t>InReview</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="G945" t="inlineStr">
@@ -69562,16 +69562,16 @@
       </c>
       <c r="Q945" t="inlineStr">
         <is>
-          <t>arman.b</t>
+          <t>not recorded</t>
         </is>
       </c>
       <c r="R945" t="inlineStr">
         <is>
-          <t>Accounting Manager</t>
+          <t>Procurement Manager</t>
         </is>
       </c>
       <c r="S945" s="5" t="n">
-        <v>46272.54395833334</v>
+        <v>46274.26350694444</v>
       </c>
     </row>
     <row r="946">
@@ -69745,7 +69745,7 @@
       </c>
       <c r="F948" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="G948" t="inlineStr">
@@ -69789,11 +69789,11 @@
       </c>
       <c r="R948" t="inlineStr">
         <is>
-          <t>Procurement Manager</t>
+          <t>LPO sent/shared with supplier</t>
         </is>
       </c>
       <c r="S948" s="5" t="n">
-        <v>46273.44671296296</v>
+        <v>46274.5</v>
       </c>
     </row>
     <row r="949">
@@ -69819,7 +69819,7 @@
       </c>
       <c r="F949" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="G949" t="inlineStr">
@@ -69863,11 +69863,11 @@
       </c>
       <c r="R949" t="inlineStr">
         <is>
-          <t>Procurement Manager</t>
+          <t>LPO sent/shared with supplier</t>
         </is>
       </c>
       <c r="S949" s="5" t="n">
-        <v>46273.44671296296</v>
+        <v>46274.5</v>
       </c>
     </row>
     <row r="950">

</xml_diff>

<commit_message>
fix: label PR prices clocks and shared buyers honestly
</commit_message>
<xml_diff>
--- a/po.xlsx
+++ b/po.xlsx
@@ -147,8 +147,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AxTable1" displayName="AxTable1" ref="A1:T997" headerRowCount="1">
-  <autoFilter ref="A1:T997"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AxTable1" displayName="AxTable1" ref="A1:T1000" headerRowCount="1">
+  <autoFilter ref="A1:T1000"/>
   <tableColumns count="20">
     <tableColumn id="1" name="Purchase order"/>
     <tableColumn id="2" name="Vendor account"/>
@@ -464,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T997"/>
+  <dimension ref="A1:T1000"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -69893,7 +69893,7 @@
       </c>
       <c r="F950" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="G950" t="inlineStr">
@@ -69937,8 +69937,11 @@
       </c>
       <c r="R950" t="inlineStr">
         <is>
-          <t>Procurement Manager</t>
-        </is>
+          <t>LPO sent/shared with supplier</t>
+        </is>
+      </c>
+      <c r="S950" s="5" t="n">
+        <v>46274.5</v>
       </c>
     </row>
     <row r="951">
@@ -70408,7 +70411,7 @@
       </c>
       <c r="F957" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="G957" t="inlineStr">
@@ -70452,11 +70455,11 @@
       </c>
       <c r="R957" t="inlineStr">
         <is>
-          <t>Procurement Manager</t>
+          <t>LPO sent/shared with supplier</t>
         </is>
       </c>
       <c r="S957" s="5" t="n">
-        <v>46273.50631944444</v>
+        <v>46274.5</v>
       </c>
     </row>
     <row r="958">
@@ -70482,7 +70485,7 @@
       </c>
       <c r="F958" t="inlineStr">
         <is>
-          <t>InReview</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="G958" t="inlineStr">
@@ -70521,16 +70524,16 @@
       </c>
       <c r="Q958" t="inlineStr">
         <is>
-          <t>Riyaz.n</t>
+          <t>not recorded</t>
         </is>
       </c>
       <c r="R958" t="inlineStr">
         <is>
-          <t>Procurement Manager</t>
+          <t>LPO sent/shared with supplier</t>
         </is>
       </c>
       <c r="S958" s="5" t="n">
-        <v>46273.54106481482</v>
+        <v>46274.5</v>
       </c>
     </row>
     <row r="959">
@@ -70556,7 +70559,7 @@
       </c>
       <c r="F959" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="G959" t="inlineStr">
@@ -70600,8 +70603,11 @@
       </c>
       <c r="R959" t="inlineStr">
         <is>
-          <t>Procurement Manager</t>
-        </is>
+          <t>LPO sent/shared with supplier</t>
+        </is>
+      </c>
+      <c r="S959" s="5" t="n">
+        <v>46274.5</v>
       </c>
     </row>
     <row r="960">
@@ -70627,7 +70633,7 @@
       </c>
       <c r="F960" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="G960" t="inlineStr">
@@ -70671,8 +70677,11 @@
       </c>
       <c r="R960" t="inlineStr">
         <is>
-          <t>Procurement Manager</t>
-        </is>
+          <t>LPO sent/shared with supplier</t>
+        </is>
+      </c>
+      <c r="S960" s="5" t="n">
+        <v>46274.5</v>
       </c>
     </row>
     <row r="961">
@@ -70698,7 +70707,7 @@
       </c>
       <c r="F961" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="G961" t="inlineStr">
@@ -70742,11 +70751,11 @@
       </c>
       <c r="R961" t="inlineStr">
         <is>
-          <t>Procurement Manager</t>
+          <t>LPO sent/shared with supplier</t>
         </is>
       </c>
       <c r="S961" s="5" t="n">
-        <v>46273.57065972222</v>
+        <v>46274.5</v>
       </c>
     </row>
     <row r="962">
@@ -70772,7 +70781,7 @@
       </c>
       <c r="F962" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="G962" t="inlineStr">
@@ -70816,11 +70825,11 @@
       </c>
       <c r="R962" t="inlineStr">
         <is>
-          <t>Procurement Manager</t>
+          <t>LPO sent/shared with supplier</t>
         </is>
       </c>
       <c r="S962" s="5" t="n">
-        <v>46273.57065972222</v>
+        <v>46274.5</v>
       </c>
     </row>
     <row r="963">
@@ -70900,27 +70909,27 @@
     <row r="964">
       <c r="A964" t="inlineStr">
         <is>
-          <t>SCPG-PO2600002</t>
+          <t>SCBM-PO2601623</t>
         </is>
       </c>
       <c r="B964" t="inlineStr">
         <is>
-          <t>VEND-00224</t>
+          <t>VEND-00762</t>
         </is>
       </c>
       <c r="C964" t="inlineStr">
         <is>
-          <t>VEND-00224</t>
+          <t>VEND-00762</t>
         </is>
       </c>
       <c r="D964" t="inlineStr">
         <is>
-          <t>Asaleeb Technology</t>
+          <t>PANACHE BUILDING MATERIALS TRADING LLC</t>
         </is>
       </c>
       <c r="F964" t="inlineStr">
         <is>
-          <t>Confirmed</t>
+          <t>Draft</t>
         </is>
       </c>
       <c r="G964" t="inlineStr">
@@ -70934,17 +70943,17 @@
         </is>
       </c>
       <c r="I964" s="5" t="n">
-        <v>46031.5</v>
+        <v>46274.5</v>
       </c>
       <c r="J964" s="5" t="n">
-        <v>46031.5</v>
+        <v>46274.5</v>
       </c>
       <c r="M964" t="n">
-        <v>2040</v>
+        <v>2412</v>
       </c>
       <c r="N964" t="inlineStr">
         <is>
-          <t>Concierge Services</t>
+          <t>Building Services</t>
         </is>
       </c>
       <c r="O964" t="inlineStr">
@@ -70964,37 +70973,34 @@
       </c>
       <c r="R964" t="inlineStr">
         <is>
-          <t>LPO sent/shared with supplier</t>
-        </is>
-      </c>
-      <c r="S964" s="5" t="n">
-        <v>46037.5</v>
+          <t>Procurement Manager</t>
+        </is>
       </c>
     </row>
     <row r="965">
       <c r="A965" t="inlineStr">
         <is>
-          <t>SCPG-PO2600004</t>
+          <t>SCBM-PO2601624</t>
         </is>
       </c>
       <c r="B965" t="inlineStr">
         <is>
-          <t>VEND-00224</t>
+          <t>VEND-00017</t>
         </is>
       </c>
       <c r="C965" t="inlineStr">
         <is>
-          <t>VEND-00224</t>
+          <t>VEND-00017</t>
         </is>
       </c>
       <c r="D965" t="inlineStr">
         <is>
-          <t>Asaleeb Technology</t>
+          <t>Eurotek Cleaning Equipment Trading LLC</t>
         </is>
       </c>
       <c r="F965" t="inlineStr">
         <is>
-          <t>Confirmed</t>
+          <t>Draft</t>
         </is>
       </c>
       <c r="G965" t="inlineStr">
@@ -71008,22 +71014,22 @@
         </is>
       </c>
       <c r="I965" s="5" t="n">
-        <v>46042.5</v>
+        <v>46274.5</v>
       </c>
       <c r="J965" s="5" t="n">
-        <v>46042.5</v>
+        <v>46274.5</v>
       </c>
       <c r="M965" t="n">
-        <v>2040</v>
+        <v>17495</v>
       </c>
       <c r="N965" t="inlineStr">
         <is>
-          <t>Accomodation Services</t>
+          <t>Contracted Cleaning Services</t>
         </is>
       </c>
       <c r="O965" t="inlineStr">
         <is>
-          <t>Al Rams</t>
+          <t>BEACH WALK 2 BY IMTIAZ</t>
         </is>
       </c>
       <c r="P965" t="inlineStr">
@@ -71038,42 +71044,39 @@
       </c>
       <c r="R965" t="inlineStr">
         <is>
-          <t>LPO sent/shared with supplier</t>
-        </is>
-      </c>
-      <c r="S965" s="5" t="n">
-        <v>46048.5</v>
+          <t>Procurement Manager</t>
+        </is>
       </c>
     </row>
     <row r="966">
       <c r="A966" t="inlineStr">
         <is>
-          <t>SCPG-PO2600005</t>
+          <t>SCBM-PO2601625</t>
         </is>
       </c>
       <c r="B966" t="inlineStr">
         <is>
-          <t>VEND-02528</t>
+          <t>VEND-00030</t>
         </is>
       </c>
       <c r="C966" t="inlineStr">
         <is>
-          <t>VEND-02528</t>
+          <t>VEND-00030</t>
         </is>
       </c>
       <c r="D966" t="inlineStr">
         <is>
-          <t>AL JABER SECURITY COMPANY L.L.C</t>
+          <t>Sharaf Dg LLC</t>
         </is>
       </c>
       <c r="F966" t="inlineStr">
         <is>
-          <t>Confirmed</t>
+          <t>Draft</t>
         </is>
       </c>
       <c r="G966" t="inlineStr">
         <is>
-          <t>Received</t>
+          <t>Backorder</t>
         </is>
       </c>
       <c r="H966" t="inlineStr">
@@ -71082,22 +71085,22 @@
         </is>
       </c>
       <c r="I966" s="5" t="n">
-        <v>46048.5</v>
+        <v>46274.5</v>
       </c>
       <c r="J966" s="5" t="n">
-        <v>46048.5</v>
+        <v>46274.5</v>
       </c>
       <c r="M966" t="n">
-        <v>52800</v>
+        <v>750</v>
       </c>
       <c r="N966" t="inlineStr">
         <is>
-          <t>Security Services</t>
+          <t>Contracted Cleaning Services</t>
         </is>
       </c>
       <c r="O966" t="inlineStr">
         <is>
-          <t>AL layyah</t>
+          <t>BEACH WALK 2 BY IMTIAZ</t>
         </is>
       </c>
       <c r="P966" t="inlineStr">
@@ -71112,32 +71115,29 @@
       </c>
       <c r="R966" t="inlineStr">
         <is>
-          <t>LPO sent/shared with supplier</t>
-        </is>
-      </c>
-      <c r="S966" s="5" t="n">
-        <v>46080.5</v>
+          <t>Procurement Manager</t>
+        </is>
       </c>
     </row>
     <row r="967">
       <c r="A967" t="inlineStr">
         <is>
-          <t>SCPG-PO2600006</t>
+          <t>SCPG-PO2600002</t>
         </is>
       </c>
       <c r="B967" t="inlineStr">
         <is>
-          <t>VEND-00465</t>
+          <t>VEND-00224</t>
         </is>
       </c>
       <c r="C967" t="inlineStr">
         <is>
-          <t>VEND-00465</t>
+          <t>VEND-00224</t>
         </is>
       </c>
       <c r="D967" t="inlineStr">
         <is>
-          <t>Fouress (Middle East) Safety Products FZC</t>
+          <t>Asaleeb Technology</t>
         </is>
       </c>
       <c r="F967" t="inlineStr">
@@ -71156,22 +71156,22 @@
         </is>
       </c>
       <c r="I967" s="5" t="n">
-        <v>46050.5</v>
+        <v>46031.5</v>
       </c>
       <c r="J967" s="5" t="n">
-        <v>46050.5</v>
+        <v>46031.5</v>
       </c>
       <c r="M967" t="n">
-        <v>210</v>
+        <v>2040</v>
       </c>
       <c r="N967" t="inlineStr">
         <is>
-          <t>Security Services</t>
+          <t>Concierge Services</t>
         </is>
       </c>
       <c r="O967" t="inlineStr">
         <is>
-          <t>THE CREEKSIDE MGALLERY HOTEL</t>
+          <t>NORTH RESIDENCE</t>
         </is>
       </c>
       <c r="P967" t="inlineStr">
@@ -71190,13 +71190,13 @@
         </is>
       </c>
       <c r="S967" s="5" t="n">
-        <v>46052.5</v>
+        <v>46037.5</v>
       </c>
     </row>
     <row r="968">
       <c r="A968" t="inlineStr">
         <is>
-          <t>SCPG-PO2600009</t>
+          <t>SCPG-PO2600004</t>
         </is>
       </c>
       <c r="B968" t="inlineStr">
@@ -71230,22 +71230,22 @@
         </is>
       </c>
       <c r="I968" s="5" t="n">
-        <v>46052.5</v>
+        <v>46042.5</v>
       </c>
       <c r="J968" s="5" t="n">
-        <v>46052.5</v>
+        <v>46042.5</v>
       </c>
       <c r="M968" t="n">
-        <v>1170</v>
+        <v>2040</v>
       </c>
       <c r="N968" t="inlineStr">
         <is>
-          <t>Concierge Services</t>
+          <t>Accomodation Services</t>
         </is>
       </c>
       <c r="O968" t="inlineStr">
         <is>
-          <t>DOMUS AL GARHOUD</t>
+          <t>Al Rams</t>
         </is>
       </c>
       <c r="P968" t="inlineStr">
@@ -71264,38 +71264,38 @@
         </is>
       </c>
       <c r="S968" s="5" t="n">
-        <v>46056.5</v>
+        <v>46048.5</v>
       </c>
     </row>
     <row r="969">
       <c r="A969" t="inlineStr">
         <is>
-          <t>SCPG-PO2600011</t>
+          <t>SCPG-PO2600005</t>
         </is>
       </c>
       <c r="B969" t="inlineStr">
         <is>
-          <t>VEND-00224</t>
+          <t>VEND-02528</t>
         </is>
       </c>
       <c r="C969" t="inlineStr">
         <is>
-          <t>VEND-00224</t>
+          <t>VEND-02528</t>
         </is>
       </c>
       <c r="D969" t="inlineStr">
         <is>
-          <t>Asaleeb Technology</t>
+          <t>AL JABER SECURITY COMPANY L.L.C</t>
         </is>
       </c>
       <c r="F969" t="inlineStr">
         <is>
-          <t>Draft</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="G969" t="inlineStr">
         <is>
-          <t>Backorder</t>
+          <t>Received</t>
         </is>
       </c>
       <c r="H969" t="inlineStr">
@@ -71304,22 +71304,22 @@
         </is>
       </c>
       <c r="I969" s="5" t="n">
-        <v>46056.5</v>
+        <v>46048.5</v>
       </c>
       <c r="J969" s="5" t="n">
-        <v>46056.5</v>
+        <v>46048.5</v>
       </c>
       <c r="M969" t="n">
-        <v>405</v>
+        <v>52800</v>
       </c>
       <c r="N969" t="inlineStr">
         <is>
-          <t>Building Services</t>
+          <t>Security Services</t>
         </is>
       </c>
       <c r="O969" t="inlineStr">
         <is>
-          <t>LE GRAND CHATEAU</t>
+          <t>AL layyah</t>
         </is>
       </c>
       <c r="P969" t="inlineStr">
@@ -71334,34 +71334,37 @@
       </c>
       <c r="R969" t="inlineStr">
         <is>
-          <t>Procurement Manager</t>
-        </is>
+          <t>LPO sent/shared with supplier</t>
+        </is>
+      </c>
+      <c r="S969" s="5" t="n">
+        <v>46080.5</v>
       </c>
     </row>
     <row r="970">
       <c r="A970" t="inlineStr">
         <is>
-          <t>SCPG-PO2600012</t>
+          <t>SCPG-PO2600006</t>
         </is>
       </c>
       <c r="B970" t="inlineStr">
         <is>
-          <t>VEND-01072</t>
+          <t>VEND-00465</t>
         </is>
       </c>
       <c r="C970" t="inlineStr">
         <is>
-          <t>VEND-01072</t>
+          <t>VEND-00465</t>
         </is>
       </c>
       <c r="D970" t="inlineStr">
         <is>
-          <t>Teclogia General Trading CO LLC</t>
+          <t>Fouress (Middle East) Safety Products FZC</t>
         </is>
       </c>
       <c r="F970" t="inlineStr">
         <is>
-          <t>Draft</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="G970" t="inlineStr">
@@ -71375,22 +71378,22 @@
         </is>
       </c>
       <c r="I970" s="5" t="n">
-        <v>46070.5</v>
+        <v>46050.5</v>
       </c>
       <c r="J970" s="5" t="n">
-        <v>46070.5</v>
+        <v>46050.5</v>
       </c>
       <c r="M970" t="n">
-        <v>5295</v>
+        <v>210</v>
       </c>
       <c r="N970" t="inlineStr">
         <is>
-          <t>Building Services</t>
+          <t>Security Services</t>
         </is>
       </c>
       <c r="O970" t="inlineStr">
         <is>
-          <t>THE PAD BY OMNIYAT</t>
+          <t>THE CREEKSIDE MGALLERY HOTEL</t>
         </is>
       </c>
       <c r="P970" t="inlineStr">
@@ -71405,29 +71408,32 @@
       </c>
       <c r="R970" t="inlineStr">
         <is>
-          <t>Procurement Manager</t>
-        </is>
+          <t>LPO sent/shared with supplier</t>
+        </is>
+      </c>
+      <c r="S970" s="5" t="n">
+        <v>46052.5</v>
       </c>
     </row>
     <row r="971">
       <c r="A971" t="inlineStr">
         <is>
-          <t>SCPG-PO2600014</t>
+          <t>SCPG-PO2600009</t>
         </is>
       </c>
       <c r="B971" t="inlineStr">
         <is>
-          <t>VEND-00216</t>
+          <t>VEND-00224</t>
         </is>
       </c>
       <c r="C971" t="inlineStr">
         <is>
-          <t>VEND-00216</t>
+          <t>VEND-00224</t>
         </is>
       </c>
       <c r="D971" t="inlineStr">
         <is>
-          <t>Arasca Medical Equipment Trading LLC</t>
+          <t>Asaleeb Technology</t>
         </is>
       </c>
       <c r="F971" t="inlineStr">
@@ -71446,22 +71452,22 @@
         </is>
       </c>
       <c r="I971" s="5" t="n">
-        <v>46105.5</v>
+        <v>46052.5</v>
       </c>
       <c r="J971" s="5" t="n">
-        <v>46105.5</v>
+        <v>46052.5</v>
       </c>
       <c r="M971" t="n">
-        <v>970.9299999999999</v>
+        <v>1170</v>
       </c>
       <c r="N971" t="inlineStr">
         <is>
-          <t>Security Services</t>
+          <t>Concierge Services</t>
         </is>
       </c>
       <c r="O971" t="inlineStr">
         <is>
-          <t>WILTON PARK RESIDENCES</t>
+          <t>DOMUS AL GARHOUD</t>
         </is>
       </c>
       <c r="P971" t="inlineStr">
@@ -71480,28 +71486,28 @@
         </is>
       </c>
       <c r="S971" s="5" t="n">
-        <v>46112.5</v>
+        <v>46056.5</v>
       </c>
     </row>
     <row r="972">
       <c r="A972" t="inlineStr">
         <is>
-          <t>SCPG-PO2600037</t>
+          <t>SCPG-PO2600011</t>
         </is>
       </c>
       <c r="B972" t="inlineStr">
         <is>
-          <t>VEND-01331</t>
+          <t>VEND-00224</t>
         </is>
       </c>
       <c r="C972" t="inlineStr">
         <is>
-          <t>VEND-01331</t>
+          <t>VEND-00224</t>
         </is>
       </c>
       <c r="D972" t="inlineStr">
         <is>
-          <t>AL MENHA TAILORING AND EMBROIDERY LLC</t>
+          <t>Asaleeb Technology</t>
         </is>
       </c>
       <c r="F972" t="inlineStr">
@@ -71520,13 +71526,13 @@
         </is>
       </c>
       <c r="I972" s="5" t="n">
-        <v>46119.5</v>
+        <v>46056.5</v>
       </c>
       <c r="J972" s="5" t="n">
-        <v>46119.5</v>
+        <v>46056.5</v>
       </c>
       <c r="M972" t="n">
-        <v>175</v>
+        <v>405</v>
       </c>
       <c r="N972" t="inlineStr">
         <is>
@@ -71535,7 +71541,7 @@
       </c>
       <c r="O972" t="inlineStr">
         <is>
-          <t>NORTH RESIDENCE</t>
+          <t>LE GRAND CHATEAU</t>
         </is>
       </c>
       <c r="P972" t="inlineStr">
@@ -71557,27 +71563,27 @@
     <row r="973">
       <c r="A973" t="inlineStr">
         <is>
-          <t>SCPG-PO2600039</t>
+          <t>SCPG-PO2600012</t>
         </is>
       </c>
       <c r="B973" t="inlineStr">
         <is>
-          <t>VEND-00216</t>
+          <t>VEND-01072</t>
         </is>
       </c>
       <c r="C973" t="inlineStr">
         <is>
-          <t>VEND-00216</t>
+          <t>VEND-01072</t>
         </is>
       </c>
       <c r="D973" t="inlineStr">
         <is>
-          <t>Arasca Medical Equipment Trading LLC</t>
+          <t>Teclogia General Trading CO LLC</t>
         </is>
       </c>
       <c r="F973" t="inlineStr">
         <is>
-          <t>Confirmed</t>
+          <t>Draft</t>
         </is>
       </c>
       <c r="G973" t="inlineStr">
@@ -71591,22 +71597,22 @@
         </is>
       </c>
       <c r="I973" s="5" t="n">
-        <v>46132.5</v>
+        <v>46070.5</v>
       </c>
       <c r="J973" s="5" t="n">
-        <v>46132.5</v>
+        <v>46070.5</v>
       </c>
       <c r="M973" t="n">
-        <v>716.59</v>
+        <v>5295</v>
       </c>
       <c r="N973" t="inlineStr">
         <is>
-          <t>Security Services</t>
+          <t>Building Services</t>
         </is>
       </c>
       <c r="O973" t="inlineStr">
         <is>
-          <t>FORTUNATO</t>
+          <t>THE PAD BY OMNIYAT</t>
         </is>
       </c>
       <c r="P973" t="inlineStr">
@@ -71621,17 +71627,14 @@
       </c>
       <c r="R973" t="inlineStr">
         <is>
-          <t>LPO sent/shared with supplier</t>
-        </is>
-      </c>
-      <c r="S973" s="5" t="n">
-        <v>46134.5</v>
+          <t>Procurement Manager</t>
+        </is>
       </c>
     </row>
     <row r="974">
       <c r="A974" t="inlineStr">
         <is>
-          <t>SCPG-PO2600040</t>
+          <t>SCPG-PO2600014</t>
         </is>
       </c>
       <c r="B974" t="inlineStr">
@@ -71665,13 +71668,13 @@
         </is>
       </c>
       <c r="I974" s="5" t="n">
-        <v>46132.5</v>
+        <v>46105.5</v>
       </c>
       <c r="J974" s="5" t="n">
-        <v>46132.5</v>
+        <v>46105.5</v>
       </c>
       <c r="M974" t="n">
-        <v>716.59</v>
+        <v>970.9299999999999</v>
       </c>
       <c r="N974" t="inlineStr">
         <is>
@@ -71680,7 +71683,7 @@
       </c>
       <c r="O974" t="inlineStr">
         <is>
-          <t>SPARKLE TOWERS</t>
+          <t>WILTON PARK RESIDENCES</t>
         </is>
       </c>
       <c r="P974" t="inlineStr">
@@ -71699,33 +71702,33 @@
         </is>
       </c>
       <c r="S974" s="5" t="n">
-        <v>46134.5</v>
+        <v>46112.5</v>
       </c>
     </row>
     <row r="975">
       <c r="A975" t="inlineStr">
         <is>
-          <t>SCPG-PO2600041</t>
+          <t>SCPG-PO2600037</t>
         </is>
       </c>
       <c r="B975" t="inlineStr">
         <is>
-          <t>VEND-00216</t>
+          <t>VEND-01331</t>
         </is>
       </c>
       <c r="C975" t="inlineStr">
         <is>
-          <t>VEND-00216</t>
+          <t>VEND-01331</t>
         </is>
       </c>
       <c r="D975" t="inlineStr">
         <is>
-          <t>Arasca Medical Equipment Trading LLC</t>
+          <t>AL MENHA TAILORING AND EMBROIDERY LLC</t>
         </is>
       </c>
       <c r="F975" t="inlineStr">
         <is>
-          <t>Confirmed</t>
+          <t>Draft</t>
         </is>
       </c>
       <c r="G975" t="inlineStr">
@@ -71739,22 +71742,22 @@
         </is>
       </c>
       <c r="I975" s="5" t="n">
-        <v>46132.5</v>
+        <v>46119.5</v>
       </c>
       <c r="J975" s="5" t="n">
-        <v>46132.5</v>
+        <v>46119.5</v>
       </c>
       <c r="M975" t="n">
-        <v>716.59</v>
+        <v>175</v>
       </c>
       <c r="N975" t="inlineStr">
         <is>
-          <t>Security Services</t>
+          <t>Building Services</t>
         </is>
       </c>
       <c r="O975" t="inlineStr">
         <is>
-          <t>SHORELINE 7AND8</t>
+          <t>NORTH RESIDENCE</t>
         </is>
       </c>
       <c r="P975" t="inlineStr">
@@ -71769,17 +71772,14 @@
       </c>
       <c r="R975" t="inlineStr">
         <is>
-          <t>LPO sent/shared with supplier</t>
-        </is>
-      </c>
-      <c r="S975" s="5" t="n">
-        <v>46134.5</v>
+          <t>Procurement Manager</t>
+        </is>
       </c>
     </row>
     <row r="976">
       <c r="A976" t="inlineStr">
         <is>
-          <t>SCPG-PO2600042</t>
+          <t>SCPG-PO2600039</t>
         </is>
       </c>
       <c r="B976" t="inlineStr">
@@ -71819,16 +71819,16 @@
         <v>46132.5</v>
       </c>
       <c r="M976" t="n">
-        <v>1175.97</v>
+        <v>716.59</v>
       </c>
       <c r="N976" t="inlineStr">
         <is>
-          <t>Leisure Services</t>
+          <t>Security Services</t>
         </is>
       </c>
       <c r="O976" t="inlineStr">
         <is>
-          <t>BALQIS RESIDENCE</t>
+          <t>FORTUNATO</t>
         </is>
       </c>
       <c r="P976" t="inlineStr">
@@ -71853,7 +71853,7 @@
     <row r="977">
       <c r="A977" t="inlineStr">
         <is>
-          <t>SCPG-PO2600043</t>
+          <t>SCPG-PO2600040</t>
         </is>
       </c>
       <c r="B977" t="inlineStr">
@@ -71893,16 +71893,16 @@
         <v>46132.5</v>
       </c>
       <c r="M977" t="n">
-        <v>1064.09</v>
+        <v>716.59</v>
       </c>
       <c r="N977" t="inlineStr">
         <is>
-          <t>Leisure Services</t>
+          <t>Security Services</t>
         </is>
       </c>
       <c r="O977" t="inlineStr">
         <is>
-          <t>SOUTH RESIDENCE</t>
+          <t>SPARKLE TOWERS</t>
         </is>
       </c>
       <c r="P977" t="inlineStr">
@@ -71927,7 +71927,7 @@
     <row r="978">
       <c r="A978" t="inlineStr">
         <is>
-          <t>SCPG-PO2600044</t>
+          <t>SCPG-PO2600041</t>
         </is>
       </c>
       <c r="B978" t="inlineStr">
@@ -71967,16 +71967,16 @@
         <v>46132.5</v>
       </c>
       <c r="M978" t="n">
-        <v>1025.45</v>
+        <v>716.59</v>
       </c>
       <c r="N978" t="inlineStr">
         <is>
-          <t>Leisure Services</t>
+          <t>Security Services</t>
         </is>
       </c>
       <c r="O978" t="inlineStr">
         <is>
-          <t>MAG 318</t>
+          <t>SHORELINE 7AND8</t>
         </is>
       </c>
       <c r="P978" t="inlineStr">
@@ -72001,7 +72001,7 @@
     <row r="979">
       <c r="A979" t="inlineStr">
         <is>
-          <t>SCPG-PO2600045</t>
+          <t>SCPG-PO2600042</t>
         </is>
       </c>
       <c r="B979" t="inlineStr">
@@ -72041,7 +72041,7 @@
         <v>46132.5</v>
       </c>
       <c r="M979" t="n">
-        <v>743.52</v>
+        <v>1175.97</v>
       </c>
       <c r="N979" t="inlineStr">
         <is>
@@ -72050,7 +72050,7 @@
       </c>
       <c r="O979" t="inlineStr">
         <is>
-          <t>THE AUTOGRAPH</t>
+          <t>BALQIS RESIDENCE</t>
         </is>
       </c>
       <c r="P979" t="inlineStr">
@@ -72075,7 +72075,7 @@
     <row r="980">
       <c r="A980" t="inlineStr">
         <is>
-          <t>SCPG-PO2600058</t>
+          <t>SCPG-PO2600043</t>
         </is>
       </c>
       <c r="B980" t="inlineStr">
@@ -72109,22 +72109,22 @@
         </is>
       </c>
       <c r="I980" s="5" t="n">
-        <v>46136.5</v>
+        <v>46132.5</v>
       </c>
       <c r="J980" s="5" t="n">
-        <v>46136.5</v>
+        <v>46132.5</v>
       </c>
       <c r="M980" t="n">
-        <v>439.6</v>
+        <v>1064.09</v>
       </c>
       <c r="N980" t="inlineStr">
         <is>
-          <t>Security Services</t>
+          <t>Leisure Services</t>
         </is>
       </c>
       <c r="O980" t="inlineStr">
         <is>
-          <t>VISTA BY PRESTIGE ONE</t>
+          <t>SOUTH RESIDENCE</t>
         </is>
       </c>
       <c r="P980" t="inlineStr">
@@ -72143,28 +72143,28 @@
         </is>
       </c>
       <c r="S980" s="5" t="n">
-        <v>46167.5</v>
+        <v>46134.5</v>
       </c>
     </row>
     <row r="981">
       <c r="A981" t="inlineStr">
         <is>
-          <t>SCPG-PO2600059</t>
+          <t>SCPG-PO2600044</t>
         </is>
       </c>
       <c r="B981" t="inlineStr">
         <is>
-          <t>VEND-01331</t>
+          <t>VEND-00216</t>
         </is>
       </c>
       <c r="C981" t="inlineStr">
         <is>
-          <t>VEND-01331</t>
+          <t>VEND-00216</t>
         </is>
       </c>
       <c r="D981" t="inlineStr">
         <is>
-          <t>AL MENHA TAILORING AND EMBROIDERY LLC</t>
+          <t>Arasca Medical Equipment Trading LLC</t>
         </is>
       </c>
       <c r="F981" t="inlineStr">
@@ -72174,7 +72174,7 @@
       </c>
       <c r="G981" t="inlineStr">
         <is>
-          <t>Received</t>
+          <t>Backorder</t>
         </is>
       </c>
       <c r="H981" t="inlineStr">
@@ -72183,22 +72183,22 @@
         </is>
       </c>
       <c r="I981" s="5" t="n">
-        <v>46146.5</v>
+        <v>46132.5</v>
       </c>
       <c r="J981" s="5" t="n">
-        <v>46146.5</v>
+        <v>46132.5</v>
       </c>
       <c r="M981" t="n">
-        <v>1456</v>
+        <v>1025.45</v>
       </c>
       <c r="N981" t="inlineStr">
         <is>
-          <t>Concierge Services</t>
+          <t>Leisure Services</t>
         </is>
       </c>
       <c r="O981" t="inlineStr">
         <is>
-          <t>BEACH WALK 1 BY IMTIAZ</t>
+          <t>MAG 318</t>
         </is>
       </c>
       <c r="P981" t="inlineStr">
@@ -72217,28 +72217,28 @@
         </is>
       </c>
       <c r="S981" s="5" t="n">
-        <v>46210.5</v>
+        <v>46134.5</v>
       </c>
     </row>
     <row r="982">
       <c r="A982" t="inlineStr">
         <is>
-          <t>SCPG-PO2600061</t>
+          <t>SCPG-PO2600045</t>
         </is>
       </c>
       <c r="B982" t="inlineStr">
         <is>
-          <t>VEND-00340</t>
+          <t>VEND-00216</t>
         </is>
       </c>
       <c r="C982" t="inlineStr">
         <is>
-          <t>VEND-00340</t>
+          <t>VEND-00216</t>
         </is>
       </c>
       <c r="D982" t="inlineStr">
         <is>
-          <t>CROWNS SECURITY SERVICES L.L.C</t>
+          <t>Arasca Medical Equipment Trading LLC</t>
         </is>
       </c>
       <c r="F982" t="inlineStr">
@@ -72248,7 +72248,7 @@
       </c>
       <c r="G982" t="inlineStr">
         <is>
-          <t>Received</t>
+          <t>Backorder</t>
         </is>
       </c>
       <c r="H982" t="inlineStr">
@@ -72257,22 +72257,22 @@
         </is>
       </c>
       <c r="I982" s="5" t="n">
-        <v>46167.5</v>
+        <v>46132.5</v>
       </c>
       <c r="J982" s="5" t="n">
-        <v>46167.5</v>
+        <v>46132.5</v>
       </c>
       <c r="M982" t="n">
-        <v>72000</v>
+        <v>743.52</v>
       </c>
       <c r="N982" t="inlineStr">
         <is>
-          <t>Concierge Services</t>
+          <t>Leisure Services</t>
         </is>
       </c>
       <c r="O982" t="inlineStr">
         <is>
-          <t>DOMUS INDIGO</t>
+          <t>THE AUTOGRAPH</t>
         </is>
       </c>
       <c r="P982" t="inlineStr">
@@ -72291,28 +72291,28 @@
         </is>
       </c>
       <c r="S982" s="5" t="n">
-        <v>1.5</v>
+        <v>46134.5</v>
       </c>
     </row>
     <row r="983">
       <c r="A983" t="inlineStr">
         <is>
-          <t>SCPG-PO2600062</t>
+          <t>SCPG-PO2600058</t>
         </is>
       </c>
       <c r="B983" t="inlineStr">
         <is>
-          <t>VEND-00207</t>
+          <t>VEND-00216</t>
         </is>
       </c>
       <c r="C983" t="inlineStr">
         <is>
-          <t>VEND-00207</t>
+          <t>VEND-00216</t>
         </is>
       </c>
       <c r="D983" t="inlineStr">
         <is>
-          <t>Apex Professional Security Services LLC</t>
+          <t>Arasca Medical Equipment Trading LLC</t>
         </is>
       </c>
       <c r="F983" t="inlineStr">
@@ -72322,7 +72322,7 @@
       </c>
       <c r="G983" t="inlineStr">
         <is>
-          <t>Received</t>
+          <t>Backorder</t>
         </is>
       </c>
       <c r="H983" t="inlineStr">
@@ -72331,13 +72331,13 @@
         </is>
       </c>
       <c r="I983" s="5" t="n">
-        <v>46190.5</v>
+        <v>46136.5</v>
       </c>
       <c r="J983" s="5" t="n">
-        <v>46190.5</v>
+        <v>46136.5</v>
       </c>
       <c r="M983" t="n">
-        <v>795000</v>
+        <v>439.6</v>
       </c>
       <c r="N983" t="inlineStr">
         <is>
@@ -72346,7 +72346,7 @@
       </c>
       <c r="O983" t="inlineStr">
         <is>
-          <t>QUEUE POINT</t>
+          <t>VISTA BY PRESTIGE ONE</t>
         </is>
       </c>
       <c r="P983" t="inlineStr">
@@ -72365,13 +72365,13 @@
         </is>
       </c>
       <c r="S983" s="5" t="n">
-        <v>46203.5</v>
+        <v>46167.5</v>
       </c>
     </row>
     <row r="984">
       <c r="A984" t="inlineStr">
         <is>
-          <t>SCPG-PO2600063</t>
+          <t>SCPG-PO2600059</t>
         </is>
       </c>
       <c r="B984" t="inlineStr">
@@ -72396,7 +72396,7 @@
       </c>
       <c r="G984" t="inlineStr">
         <is>
-          <t>Backorder</t>
+          <t>Received</t>
         </is>
       </c>
       <c r="H984" t="inlineStr">
@@ -72405,13 +72405,13 @@
         </is>
       </c>
       <c r="I984" s="5" t="n">
-        <v>46192.5</v>
+        <v>46146.5</v>
       </c>
       <c r="J984" s="5" t="n">
-        <v>46192.5</v>
+        <v>46146.5</v>
       </c>
       <c r="M984" t="n">
-        <v>306</v>
+        <v>1456</v>
       </c>
       <c r="N984" t="inlineStr">
         <is>
@@ -72420,7 +72420,7 @@
       </c>
       <c r="O984" t="inlineStr">
         <is>
-          <t>THE8</t>
+          <t>BEACH WALK 1 BY IMTIAZ</t>
         </is>
       </c>
       <c r="P984" t="inlineStr">
@@ -72439,28 +72439,28 @@
         </is>
       </c>
       <c r="S984" s="5" t="n">
-        <v>46198.5</v>
+        <v>46210.5</v>
       </c>
     </row>
     <row r="985">
       <c r="A985" t="inlineStr">
         <is>
-          <t>SCPG-PO2600065</t>
+          <t>SCPG-PO2600061</t>
         </is>
       </c>
       <c r="B985" t="inlineStr">
         <is>
-          <t>VEND-01331</t>
+          <t>VEND-00340</t>
         </is>
       </c>
       <c r="C985" t="inlineStr">
         <is>
-          <t>VEND-01331</t>
+          <t>VEND-00340</t>
         </is>
       </c>
       <c r="D985" t="inlineStr">
         <is>
-          <t>AL MENHA TAILORING AND EMBROIDERY LLC</t>
+          <t>CROWNS SECURITY SERVICES L.L.C</t>
         </is>
       </c>
       <c r="F985" t="inlineStr">
@@ -72470,7 +72470,7 @@
       </c>
       <c r="G985" t="inlineStr">
         <is>
-          <t>Backorder</t>
+          <t>Received</t>
         </is>
       </c>
       <c r="H985" t="inlineStr">
@@ -72479,22 +72479,22 @@
         </is>
       </c>
       <c r="I985" s="5" t="n">
-        <v>46204.5</v>
+        <v>46167.5</v>
       </c>
       <c r="J985" s="5" t="n">
-        <v>46204.5</v>
+        <v>46167.5</v>
       </c>
       <c r="M985" t="n">
-        <v>350</v>
+        <v>72000</v>
       </c>
       <c r="N985" t="inlineStr">
         <is>
-          <t>Contracted Cleaning Services</t>
+          <t>Concierge Services</t>
         </is>
       </c>
       <c r="O985" t="inlineStr">
         <is>
-          <t>MAG 318</t>
+          <t>DOMUS INDIGO</t>
         </is>
       </c>
       <c r="P985" t="inlineStr">
@@ -72513,28 +72513,28 @@
         </is>
       </c>
       <c r="S985" s="5" t="n">
-        <v>46220.5</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="986">
       <c r="A986" t="inlineStr">
         <is>
-          <t>SCPG-PO2600066</t>
+          <t>SCPG-PO2600062</t>
         </is>
       </c>
       <c r="B986" t="inlineStr">
         <is>
-          <t>VEND-02675</t>
+          <t>VEND-00207</t>
         </is>
       </c>
       <c r="C986" t="inlineStr">
         <is>
-          <t>VEND-02675</t>
+          <t>VEND-00207</t>
         </is>
       </c>
       <c r="D986" t="inlineStr">
         <is>
-          <t>GULF GLOBAL RESOURCES L.L.C</t>
+          <t>Apex Professional Security Services LLC</t>
         </is>
       </c>
       <c r="F986" t="inlineStr">
@@ -72544,7 +72544,7 @@
       </c>
       <c r="G986" t="inlineStr">
         <is>
-          <t>Backorder</t>
+          <t>Received</t>
         </is>
       </c>
       <c r="H986" t="inlineStr">
@@ -72553,22 +72553,22 @@
         </is>
       </c>
       <c r="I986" s="5" t="n">
-        <v>46209.5</v>
+        <v>46190.5</v>
       </c>
       <c r="J986" s="5" t="n">
-        <v>46209.5</v>
+        <v>46190.5</v>
       </c>
       <c r="M986" t="n">
-        <v>153</v>
+        <v>795000</v>
       </c>
       <c r="N986" t="inlineStr">
         <is>
-          <t>Concierge Services</t>
+          <t>Security Services</t>
         </is>
       </c>
       <c r="O986" t="inlineStr">
         <is>
-          <t>DOMUS INDIGO</t>
+          <t>QUEUE POINT</t>
         </is>
       </c>
       <c r="P986" t="inlineStr">
@@ -72587,28 +72587,28 @@
         </is>
       </c>
       <c r="S986" s="5" t="n">
-        <v>46213.5</v>
+        <v>46203.5</v>
       </c>
     </row>
     <row r="987">
       <c r="A987" t="inlineStr">
         <is>
-          <t>SCPG-PO2600067</t>
+          <t>SCPG-PO2600063</t>
         </is>
       </c>
       <c r="B987" t="inlineStr">
         <is>
-          <t>VEND-02675</t>
+          <t>VEND-01331</t>
         </is>
       </c>
       <c r="C987" t="inlineStr">
         <is>
-          <t>VEND-02675</t>
+          <t>VEND-01331</t>
         </is>
       </c>
       <c r="D987" t="inlineStr">
         <is>
-          <t>GULF GLOBAL RESOURCES L.L.C</t>
+          <t>AL MENHA TAILORING AND EMBROIDERY LLC</t>
         </is>
       </c>
       <c r="F987" t="inlineStr">
@@ -72627,13 +72627,13 @@
         </is>
       </c>
       <c r="I987" s="5" t="n">
-        <v>46209.5</v>
+        <v>46192.5</v>
       </c>
       <c r="J987" s="5" t="n">
-        <v>46209.5</v>
+        <v>46192.5</v>
       </c>
       <c r="M987" t="n">
-        <v>255</v>
+        <v>306</v>
       </c>
       <c r="N987" t="inlineStr">
         <is>
@@ -72642,7 +72642,7 @@
       </c>
       <c r="O987" t="inlineStr">
         <is>
-          <t>THE OPUS BY OMNIYAT</t>
+          <t>THE8</t>
         </is>
       </c>
       <c r="P987" t="inlineStr">
@@ -72661,28 +72661,28 @@
         </is>
       </c>
       <c r="S987" s="5" t="n">
-        <v>46210.5</v>
+        <v>46198.5</v>
       </c>
     </row>
     <row r="988">
       <c r="A988" t="inlineStr">
         <is>
-          <t>SCPG-PO2600068</t>
+          <t>SCPG-PO2600065</t>
         </is>
       </c>
       <c r="B988" t="inlineStr">
         <is>
-          <t>VEND-01125</t>
+          <t>VEND-01331</t>
         </is>
       </c>
       <c r="C988" t="inlineStr">
         <is>
-          <t>VEND-01125</t>
+          <t>VEND-01331</t>
         </is>
       </c>
       <c r="D988" t="inlineStr">
         <is>
-          <t>AMAN SECURITY AND GUARD SYSTEMS CO LLC</t>
+          <t>AL MENHA TAILORING AND EMBROIDERY LLC</t>
         </is>
       </c>
       <c r="F988" t="inlineStr">
@@ -72692,7 +72692,7 @@
       </c>
       <c r="G988" t="inlineStr">
         <is>
-          <t>Received</t>
+          <t>Backorder</t>
         </is>
       </c>
       <c r="H988" t="inlineStr">
@@ -72701,22 +72701,22 @@
         </is>
       </c>
       <c r="I988" s="5" t="n">
-        <v>46218.5</v>
+        <v>46204.5</v>
       </c>
       <c r="J988" s="5" t="n">
-        <v>46218.5</v>
+        <v>46204.5</v>
       </c>
       <c r="M988" t="n">
-        <v>663000</v>
+        <v>350</v>
       </c>
       <c r="N988" t="inlineStr">
         <is>
-          <t>Security Services</t>
+          <t>Contracted Cleaning Services</t>
         </is>
       </c>
       <c r="O988" t="inlineStr">
         <is>
-          <t>AL TAY HILLS</t>
+          <t>MAG 318</t>
         </is>
       </c>
       <c r="P988" t="inlineStr">
@@ -72735,28 +72735,28 @@
         </is>
       </c>
       <c r="S988" s="5" t="n">
-        <v>46240.5</v>
+        <v>46220.5</v>
       </c>
     </row>
     <row r="989">
       <c r="A989" t="inlineStr">
         <is>
-          <t>SCPG-PO2600069</t>
+          <t>SCPG-PO2600066</t>
         </is>
       </c>
       <c r="B989" t="inlineStr">
         <is>
-          <t>VEND-01331</t>
+          <t>VEND-02675</t>
         </is>
       </c>
       <c r="C989" t="inlineStr">
         <is>
-          <t>VEND-01331</t>
+          <t>VEND-02675</t>
         </is>
       </c>
       <c r="D989" t="inlineStr">
         <is>
-          <t>AL MENHA TAILORING AND EMBROIDERY LLC</t>
+          <t>GULF GLOBAL RESOURCES L.L.C</t>
         </is>
       </c>
       <c r="F989" t="inlineStr">
@@ -72775,13 +72775,13 @@
         </is>
       </c>
       <c r="I989" s="5" t="n">
-        <v>46219.5</v>
+        <v>46209.5</v>
       </c>
       <c r="J989" s="5" t="n">
-        <v>46219.5</v>
+        <v>46209.5</v>
       </c>
       <c r="M989" t="n">
-        <v>196</v>
+        <v>153</v>
       </c>
       <c r="N989" t="inlineStr">
         <is>
@@ -72790,7 +72790,7 @@
       </c>
       <c r="O989" t="inlineStr">
         <is>
-          <t>DOMUS AL GARHOUD</t>
+          <t>DOMUS INDIGO</t>
         </is>
       </c>
       <c r="P989" t="inlineStr">
@@ -72809,28 +72809,28 @@
         </is>
       </c>
       <c r="S989" s="5" t="n">
-        <v>46220.5</v>
+        <v>46213.5</v>
       </c>
     </row>
     <row r="990">
       <c r="A990" t="inlineStr">
         <is>
-          <t>SCPG-PO2600070</t>
+          <t>SCPG-PO2600067</t>
         </is>
       </c>
       <c r="B990" t="inlineStr">
         <is>
-          <t>VEND-01331</t>
+          <t>VEND-02675</t>
         </is>
       </c>
       <c r="C990" t="inlineStr">
         <is>
-          <t>VEND-01331</t>
+          <t>VEND-02675</t>
         </is>
       </c>
       <c r="D990" t="inlineStr">
         <is>
-          <t>AL MENHA TAILORING AND EMBROIDERY LLC</t>
+          <t>GULF GLOBAL RESOURCES L.L.C</t>
         </is>
       </c>
       <c r="F990" t="inlineStr">
@@ -72849,22 +72849,22 @@
         </is>
       </c>
       <c r="I990" s="5" t="n">
-        <v>46224.5</v>
+        <v>46209.5</v>
       </c>
       <c r="J990" s="5" t="n">
-        <v>46224.5</v>
+        <v>46209.5</v>
       </c>
       <c r="M990" t="n">
-        <v>580</v>
+        <v>255</v>
       </c>
       <c r="N990" t="inlineStr">
         <is>
-          <t>Security Services</t>
+          <t>Concierge Services</t>
         </is>
       </c>
       <c r="O990" t="inlineStr">
         <is>
-          <t>BEACH WALK 1 BY IMTIAZ</t>
+          <t>THE OPUS BY OMNIYAT</t>
         </is>
       </c>
       <c r="P990" t="inlineStr">
@@ -72883,28 +72883,28 @@
         </is>
       </c>
       <c r="S990" s="5" t="n">
-        <v>46226.5</v>
+        <v>46210.5</v>
       </c>
     </row>
     <row r="991">
       <c r="A991" t="inlineStr">
         <is>
-          <t>SCPG-PO2600071</t>
+          <t>SCPG-PO2600068</t>
         </is>
       </c>
       <c r="B991" t="inlineStr">
         <is>
-          <t>VEND-01331</t>
+          <t>VEND-01125</t>
         </is>
       </c>
       <c r="C991" t="inlineStr">
         <is>
-          <t>VEND-01331</t>
+          <t>VEND-01125</t>
         </is>
       </c>
       <c r="D991" t="inlineStr">
         <is>
-          <t>AL MENHA TAILORING AND EMBROIDERY LLC</t>
+          <t>AMAN SECURITY AND GUARD SYSTEMS CO LLC</t>
         </is>
       </c>
       <c r="F991" t="inlineStr">
@@ -72914,7 +72914,7 @@
       </c>
       <c r="G991" t="inlineStr">
         <is>
-          <t>Backorder</t>
+          <t>Received</t>
         </is>
       </c>
       <c r="H991" t="inlineStr">
@@ -72923,13 +72923,13 @@
         </is>
       </c>
       <c r="I991" s="5" t="n">
-        <v>46224.5</v>
+        <v>46218.5</v>
       </c>
       <c r="J991" s="5" t="n">
-        <v>46224.5</v>
+        <v>46218.5</v>
       </c>
       <c r="M991" t="n">
-        <v>435</v>
+        <v>663000</v>
       </c>
       <c r="N991" t="inlineStr">
         <is>
@@ -72938,7 +72938,7 @@
       </c>
       <c r="O991" t="inlineStr">
         <is>
-          <t>VISTA BY PRESTIGE ONE</t>
+          <t>AL TAY HILLS</t>
         </is>
       </c>
       <c r="P991" t="inlineStr">
@@ -72957,13 +72957,13 @@
         </is>
       </c>
       <c r="S991" s="5" t="n">
-        <v>46226.5</v>
+        <v>46240.5</v>
       </c>
     </row>
     <row r="992">
       <c r="A992" t="inlineStr">
         <is>
-          <t>SCPG-PO2600072</t>
+          <t>SCPG-PO2600069</t>
         </is>
       </c>
       <c r="B992" t="inlineStr">
@@ -72997,22 +72997,22 @@
         </is>
       </c>
       <c r="I992" s="5" t="n">
-        <v>46224.5</v>
+        <v>46219.5</v>
       </c>
       <c r="J992" s="5" t="n">
-        <v>46224.5</v>
+        <v>46219.5</v>
       </c>
       <c r="M992" t="n">
-        <v>636</v>
+        <v>196</v>
       </c>
       <c r="N992" t="inlineStr">
         <is>
-          <t>Leisure Services</t>
+          <t>Concierge Services</t>
         </is>
       </c>
       <c r="O992" t="inlineStr">
         <is>
-          <t>BEACH WALK 1 BY IMTIAZ</t>
+          <t>DOMUS AL GARHOUD</t>
         </is>
       </c>
       <c r="P992" t="inlineStr">
@@ -73031,28 +73031,28 @@
         </is>
       </c>
       <c r="S992" s="5" t="n">
-        <v>46226.5</v>
+        <v>46220.5</v>
       </c>
     </row>
     <row r="993">
       <c r="A993" t="inlineStr">
         <is>
-          <t>SCPG-PO2600073</t>
+          <t>SCPG-PO2600070</t>
         </is>
       </c>
       <c r="B993" t="inlineStr">
         <is>
-          <t>VEND-02528</t>
+          <t>VEND-01331</t>
         </is>
       </c>
       <c r="C993" t="inlineStr">
         <is>
-          <t>VEND-02528</t>
+          <t>VEND-01331</t>
         </is>
       </c>
       <c r="D993" t="inlineStr">
         <is>
-          <t>AL JABER SECURITY COMPANY L.L.C</t>
+          <t>AL MENHA TAILORING AND EMBROIDERY LLC</t>
         </is>
       </c>
       <c r="F993" t="inlineStr">
@@ -73062,7 +73062,7 @@
       </c>
       <c r="G993" t="inlineStr">
         <is>
-          <t>Received</t>
+          <t>Backorder</t>
         </is>
       </c>
       <c r="H993" t="inlineStr">
@@ -73071,13 +73071,13 @@
         </is>
       </c>
       <c r="I993" s="5" t="n">
-        <v>46239.5</v>
+        <v>46224.5</v>
       </c>
       <c r="J993" s="5" t="n">
-        <v>46239.5</v>
+        <v>46224.5</v>
       </c>
       <c r="M993" t="n">
-        <v>52800</v>
+        <v>580</v>
       </c>
       <c r="N993" t="inlineStr">
         <is>
@@ -73086,7 +73086,7 @@
       </c>
       <c r="O993" t="inlineStr">
         <is>
-          <t>AL layyah</t>
+          <t>BEACH WALK 1 BY IMTIAZ</t>
         </is>
       </c>
       <c r="P993" t="inlineStr">
@@ -73105,28 +73105,28 @@
         </is>
       </c>
       <c r="S993" s="5" t="n">
-        <v>46244.5</v>
+        <v>46226.5</v>
       </c>
     </row>
     <row r="994">
       <c r="A994" t="inlineStr">
         <is>
-          <t>SCPG-PO2600075</t>
+          <t>SCPG-PO2600071</t>
         </is>
       </c>
       <c r="B994" t="inlineStr">
         <is>
-          <t>VEND-00216</t>
+          <t>VEND-01331</t>
         </is>
       </c>
       <c r="C994" t="inlineStr">
         <is>
-          <t>VEND-00216</t>
+          <t>VEND-01331</t>
         </is>
       </c>
       <c r="D994" t="inlineStr">
         <is>
-          <t>Arasca Medical Equipment Trading LLC</t>
+          <t>AL MENHA TAILORING AND EMBROIDERY LLC</t>
         </is>
       </c>
       <c r="F994" t="inlineStr">
@@ -73145,22 +73145,22 @@
         </is>
       </c>
       <c r="I994" s="5" t="n">
-        <v>46251.5</v>
+        <v>46224.5</v>
       </c>
       <c r="J994" s="5" t="n">
-        <v>46251.5</v>
+        <v>46224.5</v>
       </c>
       <c r="M994" t="n">
-        <v>561.1900000000001</v>
+        <v>435</v>
       </c>
       <c r="N994" t="inlineStr">
         <is>
-          <t>Leisure Services</t>
+          <t>Security Services</t>
         </is>
       </c>
       <c r="O994" t="inlineStr">
         <is>
-          <t>BEACH WALK 1 BY IMTIAZ</t>
+          <t>VISTA BY PRESTIGE ONE</t>
         </is>
       </c>
       <c r="P994" t="inlineStr">
@@ -73179,13 +73179,13 @@
         </is>
       </c>
       <c r="S994" s="5" t="n">
-        <v>46266.5</v>
+        <v>46226.5</v>
       </c>
     </row>
     <row r="995">
       <c r="A995" t="inlineStr">
         <is>
-          <t>SCPG-PO2600076</t>
+          <t>SCPG-PO2600072</t>
         </is>
       </c>
       <c r="B995" t="inlineStr">
@@ -73219,22 +73219,22 @@
         </is>
       </c>
       <c r="I995" s="5" t="n">
-        <v>46260.5</v>
+        <v>46224.5</v>
       </c>
       <c r="J995" s="5" t="n">
-        <v>46260.5</v>
+        <v>46224.5</v>
       </c>
       <c r="M995" t="n">
-        <v>318</v>
+        <v>636</v>
       </c>
       <c r="N995" t="inlineStr">
         <is>
-          <t>Security Services</t>
+          <t>Leisure Services</t>
         </is>
       </c>
       <c r="O995" t="inlineStr">
         <is>
-          <t>BALQIS RESIDENCE</t>
+          <t>BEACH WALK 1 BY IMTIAZ</t>
         </is>
       </c>
       <c r="P995" t="inlineStr">
@@ -73253,38 +73253,38 @@
         </is>
       </c>
       <c r="S995" s="5" t="n">
-        <v>46266.5</v>
+        <v>46226.5</v>
       </c>
     </row>
     <row r="996">
       <c r="A996" t="inlineStr">
         <is>
-          <t>SCPG-PO2600077</t>
+          <t>SCPG-PO2600073</t>
         </is>
       </c>
       <c r="B996" t="inlineStr">
         <is>
-          <t>VEND-00689</t>
+          <t>VEND-02528</t>
         </is>
       </c>
       <c r="C996" t="inlineStr">
         <is>
-          <t>VEND-00689</t>
+          <t>VEND-02528</t>
         </is>
       </c>
       <c r="D996" t="inlineStr">
         <is>
-          <t>Microhit Technologies LLC</t>
+          <t>AL JABER SECURITY COMPANY L.L.C</t>
         </is>
       </c>
       <c r="F996" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="G996" t="inlineStr">
         <is>
-          <t>Backorder</t>
+          <t>Received</t>
         </is>
       </c>
       <c r="H996" t="inlineStr">
@@ -73293,13 +73293,13 @@
         </is>
       </c>
       <c r="I996" s="5" t="n">
-        <v>46269.5</v>
+        <v>46239.5</v>
       </c>
       <c r="J996" s="5" t="n">
-        <v>46269.5</v>
+        <v>46239.5</v>
       </c>
       <c r="M996" t="n">
-        <v>10965</v>
+        <v>52800</v>
       </c>
       <c r="N996" t="inlineStr">
         <is>
@@ -73308,7 +73308,7 @@
       </c>
       <c r="O996" t="inlineStr">
         <is>
-          <t>THE8</t>
+          <t>AL layyah</t>
         </is>
       </c>
       <c r="P996" t="inlineStr">
@@ -73323,84 +73323,306 @@
       </c>
       <c r="R996" t="inlineStr">
         <is>
-          <t>Procurement Manager</t>
+          <t>LPO sent/shared with supplier</t>
         </is>
       </c>
       <c r="S996" s="5" t="n">
-        <v>46273.2256712963</v>
+        <v>46244.5</v>
       </c>
     </row>
     <row r="997">
       <c r="A997" t="inlineStr">
         <is>
+          <t>SCPG-PO2600075</t>
+        </is>
+      </c>
+      <c r="B997" t="inlineStr">
+        <is>
+          <t>VEND-00216</t>
+        </is>
+      </c>
+      <c r="C997" t="inlineStr">
+        <is>
+          <t>VEND-00216</t>
+        </is>
+      </c>
+      <c r="D997" t="inlineStr">
+        <is>
+          <t>Arasca Medical Equipment Trading LLC</t>
+        </is>
+      </c>
+      <c r="F997" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="G997" t="inlineStr">
+        <is>
+          <t>Backorder</t>
+        </is>
+      </c>
+      <c r="H997" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="I997" s="5" t="n">
+        <v>46251.5</v>
+      </c>
+      <c r="J997" s="5" t="n">
+        <v>46251.5</v>
+      </c>
+      <c r="M997" t="n">
+        <v>561.1900000000001</v>
+      </c>
+      <c r="N997" t="inlineStr">
+        <is>
+          <t>Leisure Services</t>
+        </is>
+      </c>
+      <c r="O997" t="inlineStr">
+        <is>
+          <t>BEACH WALK 1 BY IMTIAZ</t>
+        </is>
+      </c>
+      <c r="P997" t="inlineStr">
+        <is>
+          <t>Contracted</t>
+        </is>
+      </c>
+      <c r="Q997" t="inlineStr">
+        <is>
+          <t>not recorded</t>
+        </is>
+      </c>
+      <c r="R997" t="inlineStr">
+        <is>
+          <t>LPO sent/shared with supplier</t>
+        </is>
+      </c>
+      <c r="S997" s="5" t="n">
+        <v>46266.5</v>
+      </c>
+    </row>
+    <row r="998">
+      <c r="A998" t="inlineStr">
+        <is>
+          <t>SCPG-PO2600076</t>
+        </is>
+      </c>
+      <c r="B998" t="inlineStr">
+        <is>
+          <t>VEND-01331</t>
+        </is>
+      </c>
+      <c r="C998" t="inlineStr">
+        <is>
+          <t>VEND-01331</t>
+        </is>
+      </c>
+      <c r="D998" t="inlineStr">
+        <is>
+          <t>AL MENHA TAILORING AND EMBROIDERY LLC</t>
+        </is>
+      </c>
+      <c r="F998" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="G998" t="inlineStr">
+        <is>
+          <t>Backorder</t>
+        </is>
+      </c>
+      <c r="H998" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="I998" s="5" t="n">
+        <v>46260.5</v>
+      </c>
+      <c r="J998" s="5" t="n">
+        <v>46260.5</v>
+      </c>
+      <c r="M998" t="n">
+        <v>318</v>
+      </c>
+      <c r="N998" t="inlineStr">
+        <is>
+          <t>Security Services</t>
+        </is>
+      </c>
+      <c r="O998" t="inlineStr">
+        <is>
+          <t>BALQIS RESIDENCE</t>
+        </is>
+      </c>
+      <c r="P998" t="inlineStr">
+        <is>
+          <t>Contracted</t>
+        </is>
+      </c>
+      <c r="Q998" t="inlineStr">
+        <is>
+          <t>not recorded</t>
+        </is>
+      </c>
+      <c r="R998" t="inlineStr">
+        <is>
+          <t>LPO sent/shared with supplier</t>
+        </is>
+      </c>
+      <c r="S998" s="5" t="n">
+        <v>46266.5</v>
+      </c>
+    </row>
+    <row r="999">
+      <c r="A999" t="inlineStr">
+        <is>
+          <t>SCPG-PO2600077</t>
+        </is>
+      </c>
+      <c r="B999" t="inlineStr">
+        <is>
+          <t>VEND-00689</t>
+        </is>
+      </c>
+      <c r="C999" t="inlineStr">
+        <is>
+          <t>VEND-00689</t>
+        </is>
+      </c>
+      <c r="D999" t="inlineStr">
+        <is>
+          <t>Microhit Technologies LLC</t>
+        </is>
+      </c>
+      <c r="F999" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="G999" t="inlineStr">
+        <is>
+          <t>Backorder</t>
+        </is>
+      </c>
+      <c r="H999" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="I999" s="5" t="n">
+        <v>46269.5</v>
+      </c>
+      <c r="J999" s="5" t="n">
+        <v>46269.5</v>
+      </c>
+      <c r="M999" t="n">
+        <v>10965</v>
+      </c>
+      <c r="N999" t="inlineStr">
+        <is>
+          <t>Security Services</t>
+        </is>
+      </c>
+      <c r="O999" t="inlineStr">
+        <is>
+          <t>THE8</t>
+        </is>
+      </c>
+      <c r="P999" t="inlineStr">
+        <is>
+          <t>Contracted</t>
+        </is>
+      </c>
+      <c r="Q999" t="inlineStr">
+        <is>
+          <t>not recorded</t>
+        </is>
+      </c>
+      <c r="R999" t="inlineStr">
+        <is>
+          <t>Procurement Manager</t>
+        </is>
+      </c>
+      <c r="S999" s="5" t="n">
+        <v>46273.2256712963</v>
+      </c>
+    </row>
+    <row r="1000">
+      <c r="A1000" t="inlineStr">
+        <is>
           <t>SCPG-PO2600078</t>
         </is>
       </c>
-      <c r="B997" t="inlineStr">
+      <c r="B1000" t="inlineStr">
         <is>
           <t>VEND-00689</t>
         </is>
       </c>
-      <c r="C997" t="inlineStr">
+      <c r="C1000" t="inlineStr">
         <is>
           <t>VEND-00689</t>
         </is>
       </c>
-      <c r="D997" t="inlineStr">
+      <c r="D1000" t="inlineStr">
         <is>
           <t>Microhit Technologies LLC</t>
         </is>
       </c>
-      <c r="F997" t="inlineStr">
+      <c r="F1000" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="G997" t="inlineStr">
+      <c r="G1000" t="inlineStr">
         <is>
           <t>Backorder</t>
         </is>
       </c>
-      <c r="H997" t="inlineStr">
-        <is>
-          <t>AED</t>
-        </is>
-      </c>
-      <c r="I997" s="5" t="n">
+      <c r="H1000" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="I1000" s="5" t="n">
         <v>46269.5</v>
       </c>
-      <c r="J997" s="5" t="n">
+      <c r="J1000" s="5" t="n">
         <v>46269.5</v>
       </c>
-      <c r="M997" t="n">
+      <c r="M1000" t="n">
         <v>8685</v>
       </c>
-      <c r="N997" t="inlineStr">
+      <c r="N1000" t="inlineStr">
         <is>
           <t>Security Services</t>
         </is>
       </c>
-      <c r="O997" t="inlineStr">
+      <c r="O1000" t="inlineStr">
         <is>
           <t>MOVENPICK LAGUNA</t>
         </is>
       </c>
-      <c r="P997" t="inlineStr">
+      <c r="P1000" t="inlineStr">
         <is>
           <t>Contracted</t>
         </is>
       </c>
-      <c r="Q997" t="inlineStr">
-        <is>
-          <t>not recorded</t>
-        </is>
-      </c>
-      <c r="R997" t="inlineStr">
+      <c r="Q1000" t="inlineStr">
+        <is>
+          <t>not recorded</t>
+        </is>
+      </c>
+      <c r="R1000" t="inlineStr">
         <is>
           <t>Procurement Manager</t>
         </is>
       </c>
-      <c r="S997" s="5" t="n">
+      <c r="S1000" s="5" t="n">
         <v>46273.21885416667</v>
       </c>
     </row>

</xml_diff>